<commit_message>
Parceiros: segurar o WhatsApp copia o link com mensagem e corrige célula com dois telefones
</commit_message>
<xml_diff>
--- a/scripts/empresasparceiras.xlsx
+++ b/scripts/empresasparceiras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\tr.alienigenaV5-main\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA8984F4-F6ED-4671-8476-5471C54A96D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0FBB28-5BA3-473C-BFEB-4F111D80AA15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,9 +43,6 @@
     <t>Oficina, peças, pneus, tacógrafo, troca de óleo, guincho, reboque 24 horas, munck e manutenção para veículos pesados.</t>
   </si>
   <si>
-    <t>(88) 9665-9572</t>
-  </si>
-  <si>
     <t>@tiaotruckcenter_</t>
   </si>
   <si>
@@ -185,6 +182,9 @@
   </si>
   <si>
     <t>https://www.instagram.com/autopostogatao/</t>
+  </si>
+  <si>
+    <t>(88) 99665-9572</t>
   </si>
 </sst>
 </file>
@@ -474,166 +474,166 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" t="s">
         <v>38</v>
-      </c>
-      <c r="E8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" t="s">
         <v>42</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E11" t="s">
         <v>53</v>
-      </c>
-      <c r="E11" t="s">
-        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>